<commit_message>
thay đổi vị trí các cột, mở rộng mảng cần xoá thành (10000:46)
</commit_message>
<xml_diff>
--- a/data/product_data/Thông tin sản phẩm.xlsx
+++ b/data/product_data/Thông tin sản phẩm.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\sinvoice-creator\data\product_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\sinvoice-creator\sinvoice-creator\data\product_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A523E5E4-5794-4EB6-9843-33394610BA8F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1360E8E-D708-4158-A734-7D1C36DFF33F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AD807B91-3D44-4B7C-B5DF-3904750413C2}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="258">
   <si>
     <t>Lá Kim cuốn cơm 10g*64EA (HD)</t>
   </si>
@@ -762,6 +762,51 @@
   </si>
   <si>
     <t>Cốc O’food mừng đại lễ + Ecom</t>
+  </si>
+  <si>
+    <t>1108971</t>
+  </si>
+  <si>
+    <t>Sốt thịt kho kiểu Đông Pha 80g * 60EA (HD)</t>
+  </si>
+  <si>
+    <t>1108973</t>
+  </si>
+  <si>
+    <t>Sốt trộn gỏi - nộm 80g*60EA (HD)</t>
+  </si>
+  <si>
+    <t>2150594</t>
+  </si>
+  <si>
+    <t>TPBS Nucare vị gạo rang 200ml * 30EA</t>
+  </si>
+  <si>
+    <t>6038127</t>
+  </si>
+  <si>
+    <t>Móc khóa O'Food - nhân vật Trái Cây Nhiệt Đới + MT</t>
+  </si>
+  <si>
+    <t>2150595</t>
+  </si>
+  <si>
+    <t>TPBS Nucare vị mè đen 200ml * 30EA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hộp </t>
+  </si>
+  <si>
+    <t>2153828</t>
+  </si>
+  <si>
+    <t>Thực phẩm bổ sung Nucare vị mè đen 200ml * 24EA</t>
+  </si>
+  <si>
+    <t>1025312</t>
+  </si>
+  <si>
+    <t>Lá Kim tẩm dầu Ô liu 4g lốc 3 * 24 lốc (HD)</t>
   </si>
 </sst>
 </file>
@@ -1149,7 +1194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6EAB637-782F-4865-843F-5C89801F0A39}">
-  <dimension ref="A1:E118"/>
+  <dimension ref="A1:E125"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
@@ -2811,6 +2856,104 @@
         <v>0.08</v>
       </c>
     </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>243</v>
+      </c>
+      <c r="B119" t="s">
+        <v>244</v>
+      </c>
+      <c r="C119" t="s">
+        <v>65</v>
+      </c>
+      <c r="D119" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>245</v>
+      </c>
+      <c r="B120" t="s">
+        <v>246</v>
+      </c>
+      <c r="C120" t="s">
+        <v>65</v>
+      </c>
+      <c r="D120" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>247</v>
+      </c>
+      <c r="B121" t="s">
+        <v>248</v>
+      </c>
+      <c r="C121" t="s">
+        <v>69</v>
+      </c>
+      <c r="D121" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>249</v>
+      </c>
+      <c r="B122" t="s">
+        <v>250</v>
+      </c>
+      <c r="C122" t="s">
+        <v>67</v>
+      </c>
+      <c r="D122" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>251</v>
+      </c>
+      <c r="B123" t="s">
+        <v>252</v>
+      </c>
+      <c r="C123" t="s">
+        <v>253</v>
+      </c>
+      <c r="D123" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>254</v>
+      </c>
+      <c r="B124" t="s">
+        <v>255</v>
+      </c>
+      <c r="C124" t="s">
+        <v>253</v>
+      </c>
+      <c r="D124" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>256</v>
+      </c>
+      <c r="B125" t="s">
+        <v>257</v>
+      </c>
+      <c r="C125" t="s">
+        <v>64</v>
+      </c>
+      <c r="D125" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A1048576 G1:G1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="3"/>

</xml_diff>